<commit_message>
Sync checklist, roadmap and ledger to 14 Oct 2026 degree audit
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012zoe9p2gYUKrMz8itSXJDw
</commit_message>
<xml_diff>
--- a/UoPeople_CS_Degree_Roadmap_updated.xlsx
+++ b/UoPeople_CS_Degree_Roadmap_updated.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -864,7 +864,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Completed. Accepted as MATH 1201.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Completed. Accepted as MATH 1201.</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Sophia Eng Comp I maps to ENGL 1102.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Sophia Eng Comp I maps to ENGL 1102.</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>One Sophia Python course covers both CS 1101 and CS 1102.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Counted for both CS 1101 and CS 1102. One Sophia Python course covers both CS 1101 and CS 1102.</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Same Sophia course as above – dual credit.</t>
+          <t xml:space="preserve">Posted on the UoPeople audit 14 Oct 2026. Python counted for both CS 1101 and CS 1102. </t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>DONE (not posted)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Completed. Accepted as CS 1103.</t>
+          <t>NOT posted on 14 Oct audit: CS 1103 still Not Started. On the published Sophia list, so ask the transfer office. Completed. Accepted as CS 1103.</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Completed. Accepted as CS 2203.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Completed. Accepted as CS 2203.</t>
         </is>
       </c>
     </row>
@@ -1099,12 +1099,12 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>DONE (not posted)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Public Speaking completed; covers one Social Sci GE slot.</t>
+          <t>NOT posted on 14 Oct audit. Social Science still needs 3 credits. Public Speaking completed; covers one Social Sci GE slot.</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>U.S. Government completed; covers second Social Sci GE slot.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Posted as Humanities (HIST 1020). U.S. Government completed; covers second Social Sci GE slot.</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Critical Thinking completed; covers one Humanities GE slot.</t>
+          <t>Not posted and not needed: Humanities is complete via Art History + U.S. Government. Critical Thinking completed; covers one Humanities GE slot.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Project Management = confirmed general elective.</t>
+          <t>Not posted and not needed: the General Elective posted as Nutrition. Project Management = confirmed general elective.</t>
         </is>
       </c>
     </row>
@@ -1273,12 +1273,12 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Month 1 (pair with Ethics). Direct Sophia equivalent.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Month 1 (pair with Ethics). Direct Sophia equivalent.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
         </is>
       </c>
     </row>
@@ -1313,12 +1313,12 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Month 1 (pair with Statistics). Maps to Values &amp; Ethical Reasoning GE.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Month 1 (pair with Statistics). Maps to Values &amp; Ethical Reasoning GE.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
         </is>
       </c>
     </row>
@@ -1353,12 +1353,12 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Month 2 (pair with Env Science). Confirm with advisor if 2 Social Sci slots already filled.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Month 2 (pair with Env Science). Confirm with advisor if 2 Social Sci slots already filled.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
         </is>
       </c>
     </row>
@@ -1393,12 +1393,12 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Month 2 (pair with Psychology). Fastest natural science option.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Month 2 (pair with Psychology). Fastest natural science option.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
         </is>
       </c>
     </row>
@@ -1433,12 +1433,12 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Month 3 (pair with Networking). Covers second Humanities GE slot.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Month 3 (pair with Networking). Covers second Humanities GE slot.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
         </is>
       </c>
     </row>
@@ -1473,12 +1473,12 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Month 3 (pair with Art History). Direct equivalent.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Posted as CS 2204. Month 3 (pair with Art History). Direct equivalent.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
         </is>
       </c>
     </row>
@@ -1513,12 +1513,12 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Month 4 (pair with Calculus). Proctored at UoPeople – transferring saves the exam.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Month 4 (pair with Calculus). Proctored at UoPeople – transferring saves the exam.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
         </is>
       </c>
     </row>
@@ -1553,12 +1553,12 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE (not posted)</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>Month 4 (pair with Web Programming 1). Direct Sophia equivalent.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t>NOT posted on 14 Oct audit: MATH 1211 Not Started. Confirm the Study.com transcript was submitted. Month 4 (pair with Web Programming 1). Direct Sophia equivalent.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
         </is>
       </c>
     </row>
@@ -1593,19 +1593,19 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>Month 5 (solo or pair). Swapped from Art History II: that course maps to AHIST 1401 (Humanities), not this Civilization Studies slot. Approaches to Studying Religions (Sophia) / History 101 (Study.com) map directly to the Civilization Studies requirement.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t>Posted on the UoPeople audit 14 Oct 2026. Month 5 (solo or pair). Swapped from Art History II: that course maps to AHIST 1401 (Humanities), not this Civilization Studies slot. Approaches to Studying Religions (Sophia) / History 101 (Study.com) map directly to the Civilization Studies requirement.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>── 🟠  STUDY.COM – AFTER SOPHIA  (10 courses · ~2 months · ~$470 total, 5 courses per $235 month) ──</t>
+          <t>── 🟠  STUDY.COM – AFTER SOPHIA  (9 courses · ~2 months · ~$470 total, 5 courses per $235 month) ──</t>
         </is>
       </c>
       <c r="B24" s="43" t="n"/>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>Month 1. Confirmed UoPeople transfer equivalency. Proctored at UoPeople, so transferring avoids the exam.</t>
+          <t>Month 1. Proctored at UoPeople, so transferring avoids the exam.</t>
         </is>
       </c>
     </row>
@@ -1822,17 +1822,17 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Programming 1</t>
+          <t>Professional Communication</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>CS 1102</t>
+          <t>COM 2001</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Computer Science 115</t>
+          <t>Study.com – Business 113, Business 313 or Communications 102</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>Month 2 at Study.com. Fills the CS 1102 gap: the Sophia Python course covers CS 1101 only.</t>
+          <t>Month 2 at Study.com. Fills the COM 2001 gap in the Communication GE (audit 14 Oct: Not Started).</t>
         </is>
       </c>
     </row>
@@ -1862,17 +1862,17 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Professional Communication</t>
+          <t>Software Engineering 1</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>COM 2001</t>
+          <t>CS 2401</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Business 113, Business 313 or Communications 102</t>
+          <t>Study.com – Computer Science 307: Software Engineering</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>Month 2. Fills the COM 2001 gap in the Communication GE.</t>
+          <t>Month 2. Moved from UoPeople. Needs the 75% transfer-cap exception.</t>
         </is>
       </c>
     </row>
@@ -1902,17 +1902,17 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Software Engineering 1</t>
+          <t>Elective – Systems &amp; App Security</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>CS 2401</t>
+          <t>CS 3340</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Computer Science 307: Software Engineering</t>
+          <t>Study.com – Computer Science 110: Introduction to Cybersecurity</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -1942,17 +1942,17 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Elective – Systems &amp; App Security</t>
+          <t>Elective – Artificial Intelligence</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>CS 3340</t>
+          <t>CS 4408</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Computer Science 110: Introduction to Cybersecurity</t>
+          <t>Study.com – Computer Science 311: Artificial Intelligence</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -1976,77 +1976,77 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>Elective – Artificial Intelligence</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>CS 4408</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>Study.com – Computer Science 311: Artificial Intelligence</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Study.com</t>
-        </is>
-      </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>incl.</t>
-        </is>
-      </c>
-      <c r="G34" s="8" t="inlineStr">
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>── 🟡  UOPEOPLE – MUST TAKE DIRECTLY  (11 courses · ~$1,980 in assessment fees at $180/course) ──</t>
+        </is>
+      </c>
+      <c r="B34" s="43" t="n"/>
+      <c r="C34" s="43" t="n"/>
+      <c r="D34" s="43" t="n"/>
+      <c r="E34" s="43" t="n"/>
+      <c r="F34" s="43" t="n"/>
+      <c r="G34" s="43" t="n"/>
+      <c r="H34" s="44" t="n"/>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Online Education Strategies</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>UNIV 1001</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>UoPeople – Required orientation course</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>UoPeople</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>$180</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>Month 2. Moved from UoPeople. Needs the 75% transfer-cap exception.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>── 🟡  UOPEOPLE – MUST TAKE DIRECTLY  (10 courses · ~$1,800 in assessment fees at $180/course) ──</t>
-        </is>
-      </c>
-      <c r="B35" s="43" t="n"/>
-      <c r="C35" s="43" t="n"/>
-      <c r="D35" s="43" t="n"/>
-      <c r="E35" s="43" t="n"/>
-      <c r="F35" s="43" t="n"/>
-      <c r="G35" s="43" t="n"/>
-      <c r="H35" s="44" t="n"/>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>Term 1. Required first course; not transferable.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Online Education Strategies</t>
+          <t>Web Programming 2</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>UNIV 1001</t>
+          <t>CS 3305</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>UoPeople – Required orientation course</t>
+          <t>UoPeople – No confirmed transfer equivalent</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
@@ -2066,27 +2066,27 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>Term 1. Required first course; not transferable.</t>
+          <t>Term 1. Prereq: CS 2205 (posted).</t>
         </is>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Web Programming 2</t>
+          <t>Operating Systems 2</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>CS 3305</t>
+          <t>CS 3307</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>UoPeople – No confirmed transfer equivalent</t>
+          <t>UoPeople – Study.com CS 305 also maps, but the 90-credit ceiling is full</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -2106,27 +2106,27 @@
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>Term 1. Prereq: CS 2205 (already handled via Sophia).</t>
+          <t>Term 2. Prereq: CS 2301 (Study.com).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>Operating Systems 2</t>
+          <t>Elective – Analysis of Algorithms</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>CS 3307</t>
+          <t>CS 3304</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>UoPeople – Study.com CS 305 also maps, but the 90-credit ceiling is full</t>
+          <t>UoPeople – Take after Data Structures</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
@@ -2146,27 +2146,27 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>Term 2. Prereq: CS 2301 (Study.com).</t>
+          <t>Term 2.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>Elective – Analysis of Algorithms</t>
+          <t>Comparative Programming Languages</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>CS 3304</t>
+          <t>CS 4402</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>UoPeople – Take after Data Structures</t>
+          <t>UoPeople – No confirmed transfer equivalent</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -2186,22 +2186,22 @@
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>Term 2. Natural follow-on to Data Structures.</t>
+          <t>Term 3.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>Comparative Programming Languages</t>
+          <t>Data Mining and Machine Learning</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>CS 4402</t>
+          <t>CS 4407</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -2226,27 +2226,27 @@
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>Term 3. Upper-division; take after core CS courses are done.</t>
+          <t>Term 3.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>Data Mining and Machine Learning</t>
+          <t>Elective – Advanced Networking &amp; Security</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>CS 4407</t>
+          <t>CS 4404</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>UoPeople – No confirmed transfer equivalent</t>
+          <t>UoPeople – Strong fit with GCIH/GSEC certs</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
@@ -2266,27 +2266,27 @@
       </c>
       <c r="H41" s="11" t="inlineStr">
         <is>
-          <t>Term 3. Pairs well with the AI course.</t>
+          <t>Term 4.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>Elective – Advanced Networking &amp; Security</t>
+          <t>Elective – Big Data</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>CS 4404</t>
+          <t>CS 3440</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>UoPeople – Strong fit with GCIH/GSEC certs</t>
+          <t>UoPeople</t>
         </is>
       </c>
       <c r="E42" s="10" t="inlineStr">
@@ -2312,16 +2312,16 @@
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>Elective – Big Data</t>
+          <t>Elective – Software Engineering 2</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>CS 3440</t>
+          <t>CS 4403</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
@@ -2346,22 +2346,22 @@
       </c>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>Term 4. Good pairing with ML/AI courses.</t>
+          <t>Term 5.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>Elective – Software Engineering 2</t>
+          <t>Elective – Mobile Applications</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>CS 4403</t>
+          <t>CS 4405</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -2386,22 +2386,22 @@
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>Term 5. Follow-on to Software Engineering 1.</t>
+          <t>Term 5.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>Elective – Mobile Applications</t>
+          <t>Elective – Information Retrieval</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>CS 4405</t>
+          <t>CS 3308</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="H45" s="11" t="inlineStr">
         <is>
-          <t>Term 5. Good for app/product building goals.</t>
+          <t>Term 5. Eighth Major Elective, needed because only Cybersecurity Fundamentals posted from Google IT.</t>
         </is>
       </c>
     </row>
@@ -2434,18 +2434,21 @@
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>* Sophia: $79/mo (2 courses simultaneously, self-paced)  |  Study.com: $235/mo College Saver (2 courses active at a time)  |  UoPeople: $180 assessment fee/course  |  + ~$357 UoPeople transfer processing fees ($17 × 21 transfers)  |  GRAND TOTAL remaining: ~$3,022  |  Transfer credits: 30 courses (90 credits), exactly the 75% ceiling  |  ⚠️ See "Open Questions" tab: transfer-cap approval still needs advisor confirmation</t>
-        </is>
-      </c>
-    </row>
+          <t>* Sophia: $79/mo  |  Study.com: $235/mo College Saver (2 courses active at a time)  |  UoPeople: $180 assessment fee/course  |  + ~$357 UoPeople transfer processing fees ($17 × 21)  |  GRAND TOTAL remaining: ~$3,202  |  Audit 14 Oct 2026: 51 of 120 credits posted. Plan transfers 87 credits if everything posts, under the 90-credit ceiling  |  ⚠️ See "Open Questions" tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A35:H35"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A47:H47"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2457,7 +2460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3372,17 +3375,17 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Programming 1</t>
+          <t>Professional Communication</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>CS 1102</t>
+          <t>COM 2001</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Study.com – CS 115</t>
+          <t>Study.com – Business 113 / Business 313 / Comm 102</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -3409,17 +3412,17 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Professional Communication</t>
+          <t>Software Engineering 1 (moved)</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>COM 2001</t>
+          <t>CS 2401</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Business 113 / Business 313 / Comm 102</t>
+          <t>Study.com – CS 307</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -3446,17 +3449,17 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Software Engineering 1 (moved)</t>
+          <t>Systems &amp; App Security (Elec, moved)</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>CS 2401</t>
+          <t>CS 3340</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Study.com – CS 307</t>
+          <t>Study.com – CS 110</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -3483,17 +3486,17 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Systems &amp; App Security (Elec, moved)</t>
+          <t>Artificial Intelligence (Elec, moved)</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>CS 3340</t>
+          <t>CS 4408</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Study.com – CS 110</t>
+          <t>Study.com – CS 311</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -3513,39 +3516,39 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Study.com Mo 2</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Artificial Intelligence (Elec, moved)</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>CS 4408</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>Study.com – CS 311</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Month 7</t>
-        </is>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>incl.</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>$865</t>
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>UoPeople Term 1</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Online Education Strategies</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>UNIV 1001</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>UoPeople</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Term 1 (~Mo 8)</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>$180</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>$1,045</t>
         </is>
       </c>
     </row>
@@ -3557,12 +3560,12 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Online Education Strategies</t>
+          <t>Web Programming 2</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>UNIV 1001</t>
+          <t>CS 3305</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
@@ -3572,7 +3575,7 @@
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>Term 1 (~Mo 8)</t>
+          <t>Term 1</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
@@ -3582,24 +3585,24 @@
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>$1,045</t>
+          <t>$1,225</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>UoPeople Term 1</t>
+          <t>UoPeople Term 2</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Web Programming 2</t>
+          <t>Operating Systems 2</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>CS 3305</t>
+          <t>CS 3307</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -3609,7 +3612,7 @@
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>Term 1</t>
+          <t>Term 2</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
@@ -3619,7 +3622,7 @@
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>$1,225</t>
+          <t>$1,405</t>
         </is>
       </c>
     </row>
@@ -3631,12 +3634,12 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Operating Systems 2</t>
+          <t>Analysis of Algorithms (Elec)</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>CS 3307</t>
+          <t>CS 3304</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
@@ -3656,24 +3659,24 @@
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>$1,405</t>
+          <t>$1,585</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>UoPeople Term 2</t>
+          <t>UoPeople Term 3</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Analysis of Algorithms (Elec)</t>
+          <t>Comparative Prog. Languages</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>CS 3304</t>
+          <t>CS 4402</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -3683,7 +3686,7 @@
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>Term 2</t>
+          <t>Term 3</t>
         </is>
       </c>
       <c r="F34" s="10" t="inlineStr">
@@ -3693,7 +3696,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>$1,585</t>
+          <t>$1,765</t>
         </is>
       </c>
     </row>
@@ -3705,12 +3708,12 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>Comparative Prog. Languages</t>
+          <t>Data Mining &amp; Machine Learning</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>CS 4402</t>
+          <t>CS 4407</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
@@ -3730,24 +3733,24 @@
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>$1,765</t>
+          <t>$1,945</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>UoPeople Term 3</t>
+          <t>UoPeople Term 4</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Data Mining &amp; Machine Learning</t>
+          <t>Advanced Net &amp; Security (Elec)</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>CS 4407</t>
+          <t>CS 4404</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3757,7 +3760,7 @@
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>Term 3</t>
+          <t>Term 4</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
@@ -3767,7 +3770,7 @@
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>$1,945</t>
+          <t>$2,125</t>
         </is>
       </c>
     </row>
@@ -3779,12 +3782,12 @@
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Advanced Net &amp; Security (Elec)</t>
+          <t>Big Data (Elective)</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>CS 4404</t>
+          <t>CS 3440</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
@@ -3804,24 +3807,24 @@
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>$2,125</t>
+          <t>$2,305</t>
         </is>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>UoPeople Term 4</t>
+          <t>UoPeople Term 5</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>Big Data (Elective)</t>
+          <t>Software Engineering 2 (Elec)</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>CS 3440</t>
+          <t>CS 4403</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3831,7 +3834,7 @@
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>Term 4</t>
+          <t>Term 5</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
@@ -3841,7 +3844,7 @@
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>$2,305</t>
+          <t>$2,485</t>
         </is>
       </c>
     </row>
@@ -3853,12 +3856,12 @@
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>Software Engineering 2 (Elec)</t>
+          <t>Mobile Applications (Elec)</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>CS 4403</t>
+          <t>CS 4405</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
@@ -3878,7 +3881,7 @@
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>$2,485</t>
+          <t>$2,665</t>
         </is>
       </c>
     </row>
@@ -3890,12 +3893,12 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>Mobile Applications (Elec)</t>
+          <t>Information Retrieval (Elec)</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>CS 4405</t>
+          <t>CS 3308</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3915,24 +3918,32 @@
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>$2,665</t>
-        </is>
-      </c>
-    </row>
+          <t>$2,845</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="40" t="inlineStr">
         <is>
-          <t>TOTAL COST BREAKDOWN:  Sophia ~$395 (5 mo) + Study.com ~$470 (2 mo, 10 courses) + UoPeople ~$1,800 (10 courses × $180) + Transfer fees ~$357 ($17 × 21)  =  GRAND TOTAL ~$3,022  |  Transfer credits: 30 courses (90 credits), exactly the 75% ceiling  |  ⚠️ Pending: transfer-cap exception approval (see Open Questions tab)</t>
+          <t>TOTAL COST BREAKDOWN:  Sophia ~$395 (5 mo) + Study.com ~$470 (2 mo, 9 courses) + UoPeople ~$1,980 (11 courses × $180) + Transfer fees ~$357 ($17 × 21)  =  GRAND TOTAL ~$3,202  |  Audit 14 Oct 2026: 51 of 120 credits posted. Plan transfers 87 credits if everything posts, under the 90-credit ceiling  |  ⚠️ Pending: transfer-cap exception approval (see Open Questions tab)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Note: If Sophia.com is processing assignments slowly, switch any Month 1–5 course to its Study.com equivalent (see Platform / Action column). Study.com allows only 2 active courses at a time, so clear one before starting the next. Budget 2 billing months ($470) for the 10 Study.com courses. If you finish all 10 in one month, the total drops by $235.</t>
-        </is>
-      </c>
-    </row>
+          <t>Note: If Sophia.com is processing assignments slowly, switch any Month 1–5 course to its Study.com equivalent. Study.com allows only 2 active courses at a time. Budget 2 billing months ($470) for the 9 Study.com courses. If you finish all 9 in one month, the total drops by $235.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
@@ -4105,7 +4116,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="41" t="inlineStr">
         <is>
-          <t>Study.com (2 months, 10 courses)</t>
+          <t>Study.com (2 months, 9 courses)</t>
         </is>
       </c>
       <c r="B15" s="42" t="inlineStr">
@@ -4117,12 +4128,12 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="41" t="inlineStr">
         <is>
-          <t>UoPeople (10 courses × $180)</t>
+          <t>UoPeople (11 courses × $180)</t>
         </is>
       </c>
       <c r="B16" s="42" t="inlineStr">
         <is>
-          <t>~$1,800</t>
+          <t>~$1,980</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4169,7 @@
       </c>
       <c r="B19" s="42" t="inlineStr">
         <is>
-          <t>~$3,082</t>
+          <t>~$3,262</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4241,7 @@
       </c>
       <c r="B26" s="42" t="inlineStr">
         <is>
-          <t>Default transfer cap is 50% of the degree (60 credits / 20 courses). Up to 75% (90 credits / 30 courses) requires University approval "in special cases", not automatic. The plan now transfers 30 courses (90 credits), exactly at the ceiling, so this approval is a prerequisite. UoPeople's own Study.com pathway guide lists 81 transfer credits, which also exceeds the default cap. Cite it in the request.</t>
+          <t>Default transfer cap is 50% of the degree (60 credits / 20 courses). Up to 75% (90 credits / 30 courses) requires University approval "in special cases", not automatic. The plan now transfers up to 87 credits if everything posts (30 courses is the ceiling), so this approval is a prerequisite. UoPeople's own Study.com pathway guide lists 81 transfer credits, which also exceeds the default cap. Cite it in the request.</t>
         </is>
       </c>
     </row>
@@ -4318,7 +4329,7 @@
       </c>
       <c r="B3" s="47" t="inlineStr">
         <is>
-          <t>UoPeople's default transfer allowance is 50% of the degree (60 credits / 20 courses). The 75% ceiling (90 credits / 30 courses) is only granted "in special cases". The plan now transfers 30 courses (90 credits), exactly the ceiling, after moving CS 2401, CS 3340 and CS 4408 to Study.com. UoPeople's own Study.com pathway guide (valid 2025-2026) lists 81 transfer credits and 39 UoPeople credits, which already exceeds 50%, so cite it. Ask the Transfer Evaluation contact whether the 75% exception applies BEFORE paying for the remaining Study.com courses. Any course not approved must be retaken at UoPeople ($180 each). No transfer credit beyond 90 counts, so the spare Psychology, Nutrition and extra Google IT credits are surplus.</t>
+          <t>UoPeople's default transfer allowance is 50% of the degree (60 credits / 20 courses). The 75% ceiling (90 credits / 30 courses) is only granted "in special cases". The plan now transfers up to 87 credits if everything posts (51 posted so far), after moving CS 2401, CS 3340 and CS 4408 to Study.com. UoPeople's own Study.com pathway guide (valid 2025-2026) lists 81 transfer credits and 39 UoPeople credits, which already exceeds 50%, so cite it. Ask the Transfer Evaluation contact whether the 75% exception applies BEFORE paying for the remaining Study.com courses. Any course not approved must be retaken at UoPeople ($180 each). No transfer credit beyond 90 counts, so the spare Psychology, Nutrition and extra Google IT credits are surplus.</t>
         </is>
       </c>
     </row>
@@ -4330,7 +4341,7 @@
       </c>
       <c r="B4" s="47" t="inlineStr">
         <is>
-          <t>The audit requires 120 credits: Major 60, General Education 30, Electives 30. The plan now has 40 courses: 30 transfer and 10 direct at UoPeople. The two uncovered required courses, CS 1102 (Study.com CS 115) and COM 2001 (Business 113, Business 313 or Communications 102), are added. Open items to confirm: whether Sophia Critical Thinking counts for the Humanities slot (the published Sophia list maps Ancient Greek Philosophers to PHIL 1402, not Critical Thinking), and how the remaining Google IT credits post as EXT-MAJ electives.</t>
+          <t>Audit of 14 Oct 2026: 51 of 120 credits posted (Major 24/60, General Education 21/30, Electives 6/30). CS 1102 posted because Python counted for both CS 1101 and CS 1102. Four Sophia courses did not post: Java (CS 1103, on the published Sophia list, so ask the transfer office), Public Speaking (should map to Social Science, which still needs 3 credits), Critical Thinking and Project Management (not needed). Calculus (MATH 1211) is not posted, so confirm the Study.com transcript was submitted. Still uncovered: COM 2001 (Study.com Business 113, Business 313 or Communications 102) and one Social Science course (Public Speaking if it posts, otherwise Sophia Introduction to Sociology). Only Cybersecurity Fundamentals posted from Google IT, so an eighth Major Elective (CS 3308) was added at UoPeople. Remaining: 23 courses, 12 by transfer and 11 direct.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record passed Study.com courses (Calculus, Discrete Math, Networking), College Saver Pro 3-at-a-time
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012zoe9p2gYUKrMz8itSXJDw
</commit_message>
<xml_diff>
--- a/UoPeople_CS_Degree_Roadmap_updated.xlsx
+++ b/UoPeople_CS_Degree_Roadmap_updated.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Posted on the UoPeople audit 14 Oct 2026. Posted as CS 2204. Month 3 (pair with Art History). Direct equivalent.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t xml:space="preserve">CS 2204 already posted from Google IT, so this is not needed there. Study.com CS 108 passed (92%), not transferred yet. Ask whether it can post as a Major Elective instead of CS 3308. </t>
         </is>
       </c>
     </row>
@@ -1553,12 +1553,12 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>DONE (not posted)</t>
+          <t>DONE (not transferred)</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>NOT posted on 14 Oct audit: MATH 1211 Not Started. Confirm the Study.com transcript was submitted. Month 4 (pair with Web Programming 1). Direct Sophia equivalent.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t xml:space="preserve">Study.com Math 104 passed (91%), not transferred yet. MATH 1211 is Not Started on the 14 Oct audit, so submit the transcript. </t>
         </is>
       </c>
     </row>
@@ -1647,12 +1647,12 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE (not transferred)</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>Month 1 at Study.com (pair with CS 1105). No Sophia equivalent.</t>
+          <t>Passed 97% on Study.com, not transferred yet. Submit the Study.com transcript.</t>
         </is>
       </c>
     </row>
@@ -2434,13 +2434,10 @@
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>* Sophia: $79/mo  |  Study.com: $235/mo College Saver (2 courses active at a time)  |  UoPeople: $180 assessment fee/course  |  + ~$357 UoPeople transfer processing fees ($17 × 21)  |  GRAND TOTAL remaining: ~$3,202  |  Audit 14 Oct 2026: 51 of 120 credits posted. Plan transfers 87 credits if everything posts, under the 90-credit ceiling  |  ⚠️ See "Open Questions" tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
+          <t>* Sophia: $79/mo  |  Study.com: $235/mo College Saver (College Saver Pro: 3 courses at a time)  |  UoPeople: $180 assessment fee/course  |  + ~$357 UoPeople transfer processing fees ($17 × 21)  |  GRAND TOTAL remaining: ~$3,202  |  Audit 14 Oct 2026: 51 of 120 credits posted. Plan transfers 87 credits if everything posts, under the 90-credit ceiling  |  ⚠️ See "Open Questions" tab</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A3:H3"/>
@@ -2460,7 +2457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3200,7 +3197,7 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Math 108</t>
+          <t>Study.com – Math 108 (PASSED 97%, not transferred yet)</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -3922,7 +3919,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="40" t="inlineStr">
         <is>
@@ -3933,17 +3929,10 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Note: If Sophia.com is processing assignments slowly, switch any Month 1–5 course to its Study.com equivalent. Study.com allows only 2 active courses at a time. Budget 2 billing months ($470) for the 9 Study.com courses. If you finish all 9 in one month, the total drops by $235.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
+          <t>Note: If Sophia.com is processing assignments slowly, switch any Month 1–5 course to its Study.com equivalent. Study.com College Saver Pro allows 3 active courses at a time. Budget 2 billing months ($470) for the 9 Study.com courses. If you finish all 9 in one month, the total drops by $235.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
@@ -4017,7 +4006,7 @@
       </c>
       <c r="B5" s="42" t="inlineStr">
         <is>
-          <t>Take on Study.com – $235/mo College Saver, up to 2 at a time, self-paced</t>
+          <t>Take on Study.com – $235/mo College Saver Pro, up to 3 at a time, self-paced</t>
         </is>
       </c>
     </row>
@@ -4069,7 +4058,7 @@
       </c>
       <c r="B10" s="42" t="inlineStr">
         <is>
-          <t>study.com | $235/mo (College Saver) | ACE/NCCRS | UoPeople-mapped pathway (see Study.com pathway guide) | Self-paced | 2 courses at a time</t>
+          <t>study.com | $235/mo (College Saver) | ACE/NCCRS | UoPeople-mapped pathway (see Study.com pathway guide) | Self-paced | 3 courses at a time</t>
         </is>
       </c>
     </row>
@@ -4212,12 +4201,12 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="41" t="inlineStr">
         <is>
-          <t>Take 2 Study.com courses/mo</t>
+          <t>Take 3 Study.com courses at a time</t>
         </is>
       </c>
       <c r="B24" s="42" t="inlineStr">
         <is>
-          <t>Study.com College Saver also allows 2 at a time – always pair for best value.</t>
+          <t>Study.com College Saver Pro allows 3 at a time – run 3 in parallel for best value.</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4330,7 @@
       </c>
       <c r="B4" s="47" t="inlineStr">
         <is>
-          <t>Audit of 14 Oct 2026: 51 of 120 credits posted (Major 24/60, General Education 21/30, Electives 6/30). CS 1102 posted because Python counted for both CS 1101 and CS 1102. Four Sophia courses did not post: Java (CS 1103, on the published Sophia list, so ask the transfer office), Public Speaking (should map to Social Science, which still needs 3 credits), Critical Thinking and Project Management (not needed). Calculus (MATH 1211) is not posted, so confirm the Study.com transcript was submitted. Still uncovered: COM 2001 (Study.com Business 113, Business 313 or Communications 102) and one Social Science course (Public Speaking if it posts, otherwise Sophia Introduction to Sociology). Only Cybersecurity Fundamentals posted from Google IT, so an eighth Major Elective (CS 3308) was added at UoPeople. Remaining: 23 courses, 12 by transfer and 11 direct.</t>
+          <t>Audit of 14 Oct 2026: 51 of 120 credits posted (Major 24/60, General Education 21/30, Electives 6/30). CS 1102 posted because Python counted for both CS 1101 and CS 1102. Four Sophia courses did not post: Java (CS 1103, on the published Sophia list, so ask the transfer office), Public Speaking (should map to Social Science, which still needs 3 credits), Critical Thinking and Project Management (not needed). Calculus (MATH 1211) is not posted, so confirm the Study.com transcript was submitted. Still uncovered: COM 2001 (Study.com Business 113, Business 313 or Communications 102) and one Social Science course (Public Speaking if it posts, otherwise Sophia Introduction to Sociology). Only Cybersecurity Fundamentals posted from Google IT, so an eighth Major Elective (CS 3308) was added at UoPeople. Remaining: 23 courses, 12 by transfer and 11 direct. Study.com update (14 Oct): Calculus (91%), Discrete Mathematics (97%) and Networking (92%) are passed but not transferred. CS 2204 already posted from Google IT, so Study.com Networking is a spare. If UoPeople accepts it as a Major Elective, it replaces CS 3308 ($180 saved) and the plan lands at exactly 90 transfer credits.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Group completed Study.com courses under Study.com, drop dual-platform toggles and alt hints
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012zoe9p2gYUKrMz8itSXJDw
</commit_message>
<xml_diff>
--- a/UoPeople_CS_Degree_Roadmap_updated.xlsx
+++ b/UoPeople_CS_Degree_Roadmap_updated.xlsx
@@ -1231,7 +1231,7 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>── 🔵  SOPHIA.COM / STUDY.COM – NEXT STEPS  (~4–5 months · ~$395–1,175 total — use whichever platform is faster per course) ──</t>
+          <t>── 🔵  SOPHIA.COM – NEXT STEPS  (7 courses · all completed) ──</t>
         </is>
       </c>
       <c r="B14" s="43" t="n"/>
@@ -1258,12 +1258,12 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Sophia – Introduction to Statistics   |   Study.com Alt: Statistics 101: Principles of Statistics</t>
+          <t>Sophia – Introduction to Statistics</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Sophia.com OR Study.com</t>
+          <t>Sophia.com</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Posted on the UoPeople audit 14 Oct 2026. Month 1 (pair with Ethics). Direct Sophia equivalent.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t xml:space="preserve">Posted on the UoPeople audit 14 Oct 2026. Month 1 (pair with Ethics). Direct Sophia equivalent. </t>
         </is>
       </c>
     </row>
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Sophia – Introduction to Ethics   |   Study.com Alt: Philosophy 103: Ethics – Theory &amp; Practice</t>
+          <t>Sophia – Introduction to Ethics</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Sophia.com OR Study.com</t>
+          <t>Sophia.com</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Posted on the UoPeople audit 14 Oct 2026. Month 1 (pair with Statistics). Maps to Values &amp; Ethical Reasoning GE.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t xml:space="preserve">Posted on the UoPeople audit 14 Oct 2026. Month 1 (pair with Statistics). Maps to Values &amp; Ethical Reasoning GE. </t>
         </is>
       </c>
     </row>
@@ -1338,12 +1338,12 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Sophia – Introduction to Psychology   |   Study.com Alt: Psychology 101: Intro to Psychology</t>
+          <t>Sophia – Introduction to Psychology</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Sophia.com OR Study.com</t>
+          <t>Sophia.com</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Posted on the UoPeople audit 14 Oct 2026. Month 2 (pair with Env Science). Confirm with advisor if 2 Social Sci slots already filled.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t xml:space="preserve">Posted on the UoPeople audit 14 Oct 2026. Month 2 (pair with Env Science). Confirm with advisor if 2 Social Sci slots already filled. </t>
         </is>
       </c>
     </row>
@@ -1378,12 +1378,12 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Sophia – Environmental Science   |   Study.com Alt: Environmental Science 101: Environment and Humanity</t>
+          <t>Sophia – Environmental Science</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Sophia.com OR Study.com</t>
+          <t>Sophia.com</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Posted on the UoPeople audit 14 Oct 2026. Month 2 (pair with Psychology). Fastest natural science option.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t xml:space="preserve">Posted on the UoPeople audit 14 Oct 2026. Month 2 (pair with Psychology). Fastest natural science option. </t>
         </is>
       </c>
     </row>
@@ -1418,12 +1418,12 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Sophia – Art History I   |   Study.com Alt: Art 103: History of Western Art I</t>
+          <t>Sophia – Art History I</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Sophia.com OR Study.com</t>
+          <t>Sophia.com</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Posted on the UoPeople audit 14 Oct 2026. Month 3 (pair with Networking). Covers second Humanities GE slot.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
+          <t xml:space="preserve">Posted on the UoPeople audit 14 Oct 2026. Month 3 (pair with Networking). Covers second Humanities GE slot. </t>
         </is>
       </c>
     </row>
@@ -1448,27 +1448,27 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Communications and Networking</t>
+          <t>Web Programming 1</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>CS 2204</t>
+          <t>CS 2205</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Sophia – Introduction to Networking   |   Study.com Alt: Computer Science 108: Introduction to Networking</t>
+          <t>Sophia – Introduction to Web Development</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Sophia.com OR Study.com</t>
+          <t>Sophia.com</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>incl.</t>
+          <t>$79/mo</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CS 2204 already posted from Google IT, so this is not needed there. Study.com CS 108 passed (92%), not transferred yet. Ask whether it can post as a Major Elective instead of CS 3308. </t>
+          <t xml:space="preserve">Posted on the UoPeople audit 14 Oct 2026. Month 4 (pair with Calculus). Proctored at UoPeople – transferring saves the exam. </t>
         </is>
       </c>
     </row>
@@ -1488,22 +1488,22 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Web Programming 1</t>
+          <t>Gen Ed – Civilization Studies / Culture &amp; Belief</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>CS 2205</t>
+          <t>Gen Ed</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Sophia – Introduction to Web Development   |   Study.com Alt: Computer Science 104: Intro to Web Development</t>
+          <t>Sophia – Approaches to Studying Religions (direct Civilization Studies/Culture &amp; Belief match)</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Sophia.com OR Study.com</t>
+          <t>Sophia.com</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1518,201 +1518,201 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Posted on the UoPeople audit 14 Oct 2026. Month 4 (pair with Calculus). Proctored at UoPeople – transferring saves the exam.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
+          <t xml:space="preserve">Posted on the UoPeople audit 14 Oct 2026. Month 5 (solo or pair). Swapped from Art History II: that course maps to AHIST 1401 (Humanities), not this Civilization Studies slot. Approaches to Studying Religions (Sophia) / History 101 (Study.com) map directly to the Civilization Studies requirement. </t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>── 🟠  STUDY.COM  (11 courses · 4 passed, 7 to go · ~2 months · ~$470 total) ──</t>
+        </is>
+      </c>
+      <c r="B22" s="43" t="n"/>
+      <c r="C22" s="43" t="n"/>
+      <c r="D22" s="43" t="n"/>
+      <c r="E22" s="43" t="n"/>
+      <c r="F22" s="43" t="n"/>
+      <c r="G22" s="43" t="n"/>
+      <c r="H22" s="44" t="n"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Calculus</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>MATH 1211</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Sophia – Calculus I   |   Study.com Alt: Math 104: Calculus</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Sophia.com OR Study.com</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Study.com – Math 104: Calculus</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Study.com</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>incl.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>DONE (not transferred)</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Study.com Math 104 passed (91%), not transferred yet. MATH 1211 is Not Started on the 14 Oct audit, so submit the transcript. </t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Gen Ed – Civilization Studies / Culture &amp; Belief</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Gen Ed</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Sophia – Approaches to Studying Religions (direct Civilization Studies/Culture &amp; Belief match)   |   Study.com Alt: History 101: Western Civilization I</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>Sophia.com OR Study.com</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>$79/mo</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>Posted on the UoPeople audit 14 Oct 2026. Month 5 (solo or pair). Swapped from Art History II: that course maps to AHIST 1401 (Humanities), not this Civilization Studies slot. Approaches to Studying Religions (Sophia) / History 101 (Study.com) map directly to the Civilization Studies requirement.  ⚡ Both platforms cover this course — take whichever processes faster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>── 🟠  STUDY.COM – AFTER SOPHIA  (9 courses · ~2 months · ~$470 total, 5 courses per $235 month) ──</t>
-        </is>
-      </c>
-      <c r="B24" s="43" t="n"/>
-      <c r="C24" s="43" t="n"/>
-      <c r="D24" s="43" t="n"/>
-      <c r="E24" s="43" t="n"/>
-      <c r="F24" s="43" t="n"/>
-      <c r="G24" s="43" t="n"/>
-      <c r="H24" s="44" t="n"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Passed 91% (4 semester hours). MATH 1211 is Not Started on the 14 Oct audit. Included in the transcript submitted 13 Oct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Communications and Networking</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>CS 2204</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Study.com – Computer Science 108: Introduction to Networking</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Study.com</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>incl.</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>DONE (not transferred)</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Passed 92%. CS 2204 already posted from Google IT, so this is a spare. Ask whether it can post as a Major Elective instead of CS 3308.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="A25" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Discrete Mathematics</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>MATH 1302</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Study.com – Math 108: Discrete Mathematics</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Study.com</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>$235/mo</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>incl.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>DONE (not transferred)</t>
         </is>
       </c>
-      <c r="H25" s="9" t="inlineStr">
-        <is>
-          <t>Passed 97% on Study.com, not transferred yet. Submit the Study.com transcript.</t>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Passed 97%. Not on the 13 Oct transcript, so include it in the next request.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Digital Electronics &amp; Computer Architecture</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>CS 1105</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Study.com – Computer Science 306: Computer Architecture</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="A26" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Operating Systems 1</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>CS 2301</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Study.com – Computer Science 105: Introduction to Operating Systems</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Study.com</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>incl.</t>
         </is>
       </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="H26" s="9" t="inlineStr">
-        <is>
-          <t>Month 1 at Study.com (pair with Discrete Math). No Sophia equivalent.</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>DONE (not transferred)</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Passed. Include it in the next request. Proctored at UoPeople.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Data Structures</t>
+          <t>Digital Electronics &amp; Computer Architecture</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>CS 3303</t>
+          <t>CS 1105</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Computer Science 201: Data Structures &amp; Algorithms</t>
+          <t>Study.com – Computer Science 306: Computer Architecture</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>incl.</t>
+          <t>$235/mo</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -1732,27 +1732,27 @@
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>Month 1. Proctored at UoPeople, so transferring avoids the exam.</t>
+          <t>Month 1 at Study.com. No Sophia equivalent.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Databases 2</t>
+          <t>Data Structures</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>CS 3306</t>
+          <t>CS 3303</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Computer Science 303: Database Management</t>
+          <t>Study.com – Computer Science 201: Data Structures &amp; Algorithms</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1772,27 +1772,27 @@
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>Month 1. Per the UoPeople/Study.com pathway guide.</t>
+          <t>Month 1. Proctored at UoPeople, so transferring avoids the exam.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Operating Systems 1</t>
+          <t>Databases 2</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>CS 2301</t>
+          <t>CS 3306</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Computer Science 105: Introduction to Operating Systems</t>
+          <t>Study.com – Computer Science 303: Database Management</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -1818,7 +1818,7 @@
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
@@ -1976,8 +1976,8 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>── 🟡  UOPEOPLE – MUST TAKE DIRECTLY  (11 courses · ~$1,980 in assessment fees at $180/course) ──</t>
         </is>
@@ -2441,10 +2441,10 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A47:H47"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A22:H22"/>
     <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>Sophia.com  →  Study.com Alt: Statistics 101: Principles of Statistics</t>
+          <t>Sophia.com</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>Sophia.com (simultaneously)  →  Study.com Alt: Philosophy 103: Ethics – Theory &amp; Practice</t>
+          <t>Sophia.com</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -2921,335 +2921,335 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Sophia Mo 2</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Intro to Psychology (Social Sci GE)</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>Gen Ed</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
-        <is>
-          <t>Sophia.com  →  Study.com Alt: Psychology 101: Intro to Psychology</t>
-        </is>
-      </c>
-      <c r="E14" s="16" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Sophia.com</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>$79</t>
         </is>
       </c>
-      <c r="G14" s="16" t="inlineStr">
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>$158</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Sophia Mo 2</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Environmental Science (Nat Sci GE)</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>Gen Ed</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
-        <is>
-          <t>Sophia.com (simultaneously)  →  Study.com Alt: Environmental Science 101: Environment and Humanity</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Sophia.com</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>incl.</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr">
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>$158</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Sophia Mo 3</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Art History I (Humanities GE 2)</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>Gen Ed</t>
         </is>
       </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>Sophia.com  →  Study.com Alt: Art 103: History of Western Art I</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Sophia.com</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Month 3</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>$79</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="G16" s="14" t="inlineStr">
         <is>
           <t>$237</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Sophia Mo 3</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Sophia Mo 4</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Web Programming 1</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>CS 2205</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>Sophia.com</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Month 4</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>$79</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>$316</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Sophia Mo 5</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Civilization Studies GE</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Gen Ed</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Sophia.com – Approaches to Studying Religions</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>Month 5</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>$79</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>$395</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Calculus</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>MATH 1211</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Study.com – Math 104 (passed 91%, not transferred)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>$395</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Communications &amp; Networking</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>CS 2204</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Sophia.com (simultaneously)  →  Study.com Alt: Computer Science 108: Introduction to Networking</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Month 3</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>incl.</t>
-        </is>
-      </c>
-      <c r="G17" s="18" t="inlineStr">
-        <is>
-          <t>$237</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t>Sophia Mo 4</t>
-        </is>
-      </c>
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <t>Web Programming 1</t>
-        </is>
-      </c>
-      <c r="C18" s="21" t="inlineStr">
-        <is>
-          <t>CS 2205</t>
-        </is>
-      </c>
-      <c r="D18" s="21" t="inlineStr">
-        <is>
-          <t>Sophia.com  →  Study.com Alt: Computer Science 104: Intro to Web Development</t>
-        </is>
-      </c>
-      <c r="E18" s="20" t="inlineStr">
-        <is>
-          <t>Month 4</t>
-        </is>
-      </c>
-      <c r="F18" s="20" t="inlineStr">
-        <is>
-          <t>$79</t>
-        </is>
-      </c>
-      <c r="G18" s="20" t="inlineStr">
-        <is>
-          <t>$316</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
-        <is>
-          <t>Sophia Mo 4</t>
-        </is>
-      </c>
-      <c r="B19" s="21" t="inlineStr">
-        <is>
-          <t>Calculus I</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>MATH 1211</t>
-        </is>
-      </c>
-      <c r="D19" s="21" t="inlineStr">
-        <is>
-          <t>Sophia.com (simultaneously)  →  Study.com Alt: Math 104: Calculus</t>
-        </is>
-      </c>
-      <c r="E19" s="20" t="inlineStr">
-        <is>
-          <t>Month 4</t>
-        </is>
-      </c>
-      <c r="F19" s="20" t="inlineStr">
-        <is>
-          <t>incl.</t>
-        </is>
-      </c>
-      <c r="G19" s="20" t="inlineStr">
-        <is>
-          <t>$316</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>Sophia Mo 5</t>
-        </is>
-      </c>
-      <c r="B20" s="23" t="inlineStr">
-        <is>
-          <t>Civilization Studies GE</t>
-        </is>
-      </c>
-      <c r="C20" s="23" t="inlineStr">
-        <is>
-          <t>Gen Ed</t>
-        </is>
-      </c>
-      <c r="D20" s="23" t="inlineStr">
-        <is>
-          <t>Sophia.com – Approaches to Studying Religions  →  Study.com Alt: History 101: Western Civilization I</t>
-        </is>
-      </c>
-      <c r="E20" s="22" t="inlineStr">
-        <is>
-          <t>Month 5</t>
-        </is>
-      </c>
-      <c r="F20" s="22" t="inlineStr">
-        <is>
-          <t>$79</t>
-        </is>
-      </c>
-      <c r="G20" s="22" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Study.com – CS 108 (passed 92%, spare)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>$395</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Study.com Mo 1</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Discrete Mathematics</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>MATH 1302</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Study.com – Math 108 (PASSED 97%, not transferred yet)</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Month 6</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>$235</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>$630</t>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Study.com – Math 108 (passed 97%, not transferred)</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>$395</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Study.com Mo 1</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Digital Electronics &amp; Arch.</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>CS 1105</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Study.com – CS 306 (simultaneously)</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Month 6</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>incl.</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>$630</t>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Operating Systems 1</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>CS 2301</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Study.com – CS 105 (passed, not transferred)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>$395</t>
         </is>
       </c>
     </row>
@@ -3261,17 +3261,17 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Data Structures</t>
+          <t>Digital Electronics &amp; Arch.</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>CS 3303</t>
+          <t>CS 1105</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Study.com – CS 201</t>
+          <t>Study.com – CS 306</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>incl.</t>
+          <t>$235</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -3298,17 +3298,17 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Databases 2</t>
+          <t>Data Structures</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>CS 3306</t>
+          <t>CS 3303</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Study.com – CS 303 (simultaneously)</t>
+          <t>Study.com – CS 201</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -3335,17 +3335,17 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Operating Systems 1</t>
+          <t>Databases 2</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>CS 2301</t>
+          <t>CS 3306</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Study.com – CS 105</t>
+          <t>Study.com – CS 303</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -3919,17 +3919,18 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="40" t="inlineStr">
         <is>
-          <t>TOTAL COST BREAKDOWN:  Sophia ~$395 (5 mo) + Study.com ~$470 (2 mo, 9 courses) + UoPeople ~$1,980 (11 courses × $180) + Transfer fees ~$357 ($17 × 21)  =  GRAND TOTAL ~$3,202  |  Audit 14 Oct 2026: 51 of 120 credits posted. Plan transfers 87 credits if everything posts, under the 90-credit ceiling  |  ⚠️ Pending: transfer-cap exception approval (see Open Questions tab)</t>
+          <t>TOTAL COST BREAKDOWN:  Sophia ~$395 (5 mo) + Study.com ~$470 (2 mo, 7 remaining courses) + UoPeople ~$1,980 (11 courses × $180) + Transfer fees ~$357 ($17 × 21)  =  GRAND TOTAL ~$3,202  |  Audit 14 Oct 2026: 51 of 120 credits posted. Plan transfers 87 credits if everything posts, under the 90-credit ceiling  |  ⚠️ Pending: transfer-cap exception approval (see Open Questions tab)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Note: If Sophia.com is processing assignments slowly, switch any Month 1–5 course to its Study.com equivalent. Study.com College Saver Pro allows 3 active courses at a time. Budget 2 billing months ($470) for the 9 Study.com courses. If you finish all 9 in one month, the total drops by $235.</t>
+          <t>Note: Study.com College Saver Pro allows 3 active courses at a time. Budget 2 billing months ($470) for the 7 remaining Study.com courses. If you finish all 9 in one month, the total drops by $235.</t>
         </is>
       </c>
     </row>
@@ -4105,7 +4106,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="41" t="inlineStr">
         <is>
-          <t>Study.com (2 months, 9 courses)</t>
+          <t>Study.com (2 months, 7 remaining courses)</t>
         </is>
       </c>
       <c r="B15" s="42" t="inlineStr">

</xml_diff>

<commit_message>
Sync to 20 Oct audit: 57 credits, Networking posted as EXT-MAJ 1002, drop CS 3308
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012zoe9p2gYUKrMz8itSXJDw
</commit_message>
<xml_diff>
--- a/UoPeople_CS_Degree_Roadmap_updated.xlsx
+++ b/UoPeople_CS_Degree_Roadmap_updated.xlsx
@@ -1525,7 +1525,7 @@
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>── 🟠  STUDY.COM  (11 courses · 4 passed, 7 to go · ~2 months · ~$470 total) ──</t>
+          <t>── 🟠  STUDY.COM  (11 courses · 4 passed, 2 posted · ~2 months · ~$470 total) ──</t>
         </is>
       </c>
       <c r="B22" s="43" t="n"/>
@@ -1567,12 +1567,12 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>DONE (not transferred)</t>
+          <t>DONE (posted)</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Passed 91% (4 semester hours). MATH 1211 is Not Started on the 14 Oct audit. Included in the transcript submitted 13 Oct.</t>
+          <t>Passed 91% (4 semester hours). Posted 21 Oct as MATH 1211 for 3 credits.</t>
         </is>
       </c>
     </row>
@@ -1607,12 +1607,12 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>DONE (not transferred)</t>
+          <t>DONE (posted)</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Passed 92%. CS 2204 already posted from Google IT, so this is a spare. Ask whether it can post as a Major Elective instead of CS 3308.</t>
+          <t>Passed 92%. Posted 21 Oct as Major Elective 2 (EXT-MAJ 1002). CS 2204 had already posted from Google IT, so CS 3308 is no longer needed.</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1979,7 @@
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>── 🟡  UOPEOPLE – MUST TAKE DIRECTLY  (11 courses · ~$1,980 in assessment fees at $180/course) ──</t>
+          <t>── 🟡  UOPEOPLE – MUST TAKE DIRECTLY  (10 courses · ~$1,800 in assessment fees at $180/course) ──</t>
         </is>
       </c>
       <c r="B34" s="43" t="n"/>
@@ -2390,51 +2390,12 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="28" customHeight="1">
-      <c r="A45" s="10" t="n">
-        <v>11</v>
-      </c>
-      <c r="B45" s="11" t="inlineStr">
-        <is>
-          <t>Elective – Information Retrieval</t>
-        </is>
-      </c>
-      <c r="C45" s="11" t="inlineStr">
-        <is>
-          <t>CS 3308</t>
-        </is>
-      </c>
-      <c r="D45" s="11" t="inlineStr">
-        <is>
-          <t>UoPeople</t>
-        </is>
-      </c>
-      <c r="E45" s="10" t="inlineStr">
-        <is>
-          <t>UoPeople</t>
-        </is>
-      </c>
-      <c r="F45" s="10" t="inlineStr">
-        <is>
-          <t>$180</t>
-        </is>
-      </c>
-      <c r="G45" s="10" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="H45" s="11" t="inlineStr">
-        <is>
-          <t>Term 5. Eighth Major Elective, needed because only Cybersecurity Fundamentals posted from Google IT.</t>
-        </is>
-      </c>
-    </row>
+    <row r="45" ht="28" customHeight="1"/>
     <row r="46" ht="14" customHeight="1"/>
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>* Sophia: $79/mo  |  Study.com: $235/mo College Saver (College Saver Pro: 3 courses at a time)  |  UoPeople: $180 assessment fee/course  |  + ~$357 UoPeople transfer processing fees ($17 × 21)  |  GRAND TOTAL remaining: ~$3,202  |  Audit 14 Oct 2026: 51 of 120 credits posted. Plan transfers 87 credits if everything posts, under the 90-credit ceiling  |  ⚠️ See "Open Questions" tab</t>
+          <t>* Sophia: $79/mo  |  Study.com: $235/mo College Saver (College Saver Pro: 3 courses at a time)  |  UoPeople: $180 assessment fee/course  |  + ~$357 UoPeople transfer processing fees ($17 × 21)  |  GRAND TOTAL remaining: ~$3,022  |  Audit 20 Oct 2026: 57 of 120 credits posted. Plan transfers 90 credits if everything posts, exactly the ceiling  |  ⚠️ See "Open Questions" tab</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3084,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Study.com – Math 104 (passed 91%, not transferred)</t>
+          <t>Study.com – Math 104 (posted as MATH 1211)</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -3160,7 +3121,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Study.com – CS 108 (passed 92%, spare)</t>
+          <t>Study.com – CS 108 (posted as EXT-MAJ 1002)</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -3882,48 +3843,12 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>UoPeople Term 5</t>
-        </is>
-      </c>
-      <c r="B40" s="11" t="inlineStr">
-        <is>
-          <t>Information Retrieval (Elec)</t>
-        </is>
-      </c>
-      <c r="C40" s="11" t="inlineStr">
-        <is>
-          <t>CS 3308</t>
-        </is>
-      </c>
-      <c r="D40" s="11" t="inlineStr">
-        <is>
-          <t>UoPeople</t>
-        </is>
-      </c>
-      <c r="E40" s="10" t="inlineStr">
-        <is>
-          <t>Term 5</t>
-        </is>
-      </c>
-      <c r="F40" s="10" t="inlineStr">
-        <is>
-          <t>$180</t>
-        </is>
-      </c>
-      <c r="G40" s="10" t="inlineStr">
-        <is>
-          <t>$2,845</t>
-        </is>
-      </c>
-    </row>
+    <row r="40" ht="22" customHeight="1"/>
     <row r="41"/>
     <row r="42">
       <c r="A42" s="40" t="inlineStr">
         <is>
-          <t>TOTAL COST BREAKDOWN:  Sophia ~$395 (5 mo) + Study.com ~$470 (2 mo, 7 remaining courses) + UoPeople ~$1,980 (11 courses × $180) + Transfer fees ~$357 ($17 × 21)  =  GRAND TOTAL ~$3,202  |  Audit 14 Oct 2026: 51 of 120 credits posted. Plan transfers 87 credits if everything posts, under the 90-credit ceiling  |  ⚠️ Pending: transfer-cap exception approval (see Open Questions tab)</t>
+          <t>TOTAL COST BREAKDOWN:  Sophia ~$395 (5 mo) + Study.com ~$470 (2 mo, 7 remaining courses) + UoPeople ~$1,800 (10 courses × $180) + Transfer fees ~$357 ($17 × 21)  =  GRAND TOTAL ~$3,022  |  Audit 20 Oct 2026: 57 of 120 credits posted. Plan transfers 90 credits if everything posts, exactly the ceiling  |  ⚠️ Pending: transfer-cap exception approval (see Open Questions tab)</t>
         </is>
       </c>
     </row>
@@ -4118,12 +4043,12 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="41" t="inlineStr">
         <is>
-          <t>UoPeople (11 courses × $180)</t>
+          <t>UoPeople (10 courses × $180)</t>
         </is>
       </c>
       <c r="B16" s="42" t="inlineStr">
         <is>
-          <t>~$1,980</t>
+          <t>~$1,800</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4084,7 @@
       </c>
       <c r="B19" s="42" t="inlineStr">
         <is>
-          <t>~$3,262</t>
+          <t>~$3,082</t>
         </is>
       </c>
     </row>
@@ -4231,7 +4156,7 @@
       </c>
       <c r="B26" s="42" t="inlineStr">
         <is>
-          <t>Default transfer cap is 50% of the degree (60 credits / 20 courses). Up to 75% (90 credits / 30 courses) requires University approval "in special cases", not automatic. The plan now transfers up to 87 credits if everything posts (30 courses is the ceiling), so this approval is a prerequisite. UoPeople's own Study.com pathway guide lists 81 transfer credits, which also exceeds the default cap. Cite it in the request.</t>
+          <t>Default transfer cap is 50% of the degree (60 credits / 20 courses). Up to 75% (90 credits / 30 courses) requires University approval "in special cases", not automatic. The plan now transfers up to 90 credits if everything posts, exactly the ceiling, so this approval is a prerequisite. UoPeople's own Study.com pathway guide lists 81 transfer credits, which also exceeds the default cap. Cite it in the request.</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4244,7 @@
       </c>
       <c r="B3" s="47" t="inlineStr">
         <is>
-          <t>UoPeople's default transfer allowance is 50% of the degree (60 credits / 20 courses). The 75% ceiling (90 credits / 30 courses) is only granted "in special cases". The plan now transfers up to 87 credits if everything posts (51 posted so far), after moving CS 2401, CS 3340 and CS 4408 to Study.com. UoPeople's own Study.com pathway guide (valid 2025-2026) lists 81 transfer credits and 39 UoPeople credits, which already exceeds 50%, so cite it. Ask the Transfer Evaluation contact whether the 75% exception applies BEFORE paying for the remaining Study.com courses. Any course not approved must be retaken at UoPeople ($180 each). No transfer credit beyond 90 counts, so the spare Psychology, Nutrition and extra Google IT credits are surplus.</t>
+          <t>UoPeople's default transfer allowance is 50% of the degree (60 credits / 20 courses). The 75% ceiling (90 credits / 30 courses) is only granted "in special cases". The plan now transfers up to 90 credits if everything posts (57 posted so far), after moving CS 2401, CS 3340 and CS 4408 to Study.com. UoPeople's own Study.com pathway guide (valid 2025-2026) lists 81 transfer credits and 39 UoPeople credits, which already exceeds 50%, so cite it. Ask the Transfer Evaluation contact whether the 75% exception applies BEFORE paying for the remaining Study.com courses. Any course not approved must be retaken at UoPeople ($180 each). No transfer credit beyond 90 counts, so the spare Psychology, Nutrition and extra Google IT credits are surplus.</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4256,7 @@
       </c>
       <c r="B4" s="47" t="inlineStr">
         <is>
-          <t>Audit of 14 Oct 2026: 51 of 120 credits posted (Major 24/60, General Education 21/30, Electives 6/30). CS 1102 posted because Python counted for both CS 1101 and CS 1102. Four Sophia courses did not post: Java (CS 1103, on the published Sophia list, so ask the transfer office), Public Speaking (should map to Social Science, which still needs 3 credits), Critical Thinking and Project Management (not needed). Calculus (MATH 1211) is not posted, so confirm the Study.com transcript was submitted. Still uncovered: COM 2001 (Study.com Business 113, Business 313 or Communications 102) and one Social Science course (Public Speaking if it posts, otherwise Sophia Introduction to Sociology). Only Cybersecurity Fundamentals posted from Google IT, so an eighth Major Elective (CS 3308) was added at UoPeople. Remaining: 23 courses, 12 by transfer and 11 direct. Study.com update (14 Oct): Calculus (91%), Discrete Mathematics (97%) and Networking (92%) are passed but not transferred. CS 2204 already posted from Google IT, so Study.com Networking is a spare. If UoPeople accepts it as a Major Elective, it replaces CS 3308 ($180 saved) and the plan lands at exactly 90 transfer credits.</t>
+          <t>Audit of 20 Oct 2026: 57 of 120 credits posted (Major 27/60, General Education 21/30, Electives 9/30). Calculus posted as MATH 1211 (3 of 4 semester hours) and Study.com Networking posted as Major Elective 2 (EXT-MAJ 1002), so CS 3308 is no longer needed. Still not posted: Java (CS 1103, on the published Sophia list, so ask the transfer office) and Public Speaking (Social Science needs 3 credits). Critical Thinking and Project Management are not needed. Discrete Mathematics and Operating Systems 1 are passed and go in the next Study.com request. Still uncovered: COM 2001 (Study.com Business 113, Business 313 or Communications 102) and one Social Science course (Public Speaking if it posts, otherwise Sophia Introduction to Sociology). Remaining: 21 courses, 11 by transfer and 10 direct. The plan lands at exactly 90 transfer credits, so there is no room for an extra transfer course.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move CS 3307 to Study.com (proctored), move CS 4408 back to UoPeople
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012zoe9p2gYUKrMz8itSXJDw
</commit_message>
<xml_diff>
--- a/UoPeople_CS_Degree_Roadmap_updated.xlsx
+++ b/UoPeople_CS_Degree_Roadmap_updated.xlsx
@@ -1942,17 +1942,17 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Elective – Artificial Intelligence</t>
+          <t>Operating Systems 2</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>CS 4408</t>
+          <t>CS 3307</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Study.com – Computer Science 311: Artificial Intelligence</t>
+          <t>Study.com – Computer Science 305: Operating Systems</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>Month 2. Moved from UoPeople. Needs the 75% transfer-cap exception.</t>
+          <t>Month 2. Proctored at UoPeople, so transferring avoids the exam. Needs the 75% transfer-cap room.</t>
         </is>
       </c>
     </row>
@@ -2076,17 +2076,17 @@
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Operating Systems 2</t>
+          <t>Elective – Artificial Intelligence</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>CS 3307</t>
+          <t>CS 4408</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>UoPeople – Study.com CS 305 also maps, but the 90-credit ceiling is full</t>
+          <t>UoPeople – Moved back from Study.com to make room for CS 3307</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>Term 2. Prereq: CS 2301 (Study.com).</t>
+          <t>Term 2. Pairs well with Data Mining &amp; Machine Learning.</t>
         </is>
       </c>
     </row>
@@ -3444,17 +3444,17 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Artificial Intelligence (Elec, moved)</t>
+          <t>Operating Systems 2 (proctored)</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>CS 4408</t>
+          <t>CS 3307</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Study.com – CS 311</t>
+          <t>Study.com – CS 305</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -3555,12 +3555,12 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Operating Systems 2</t>
+          <t>Artificial Intelligence (Elec)</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>CS 3307</t>
+          <t>CS 4408</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="B25" s="42" t="inlineStr">
         <is>
-          <t>CS 3303 (Data Structures) and CS 2205 (Web Programming 1) are proctored at UoPeople. Transferring via Study.com/Sophia avoids those exams.</t>
+          <t>Proctored courses (8 required): CS 2205, MATH 1201 and MATH 1280 are posted. Study.com covers CS 2301, 3303, 3306 and 3307 so you skip those exams. CS 3305, 4402 and 4407 have no transfer equivalent, so you take those 3 proctored exams at UoPeople.</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="B3" s="47" t="inlineStr">
         <is>
-          <t>UoPeople's default transfer allowance is 50% of the degree (60 credits / 20 courses). The 75% ceiling (90 credits / 30 courses) is only granted "in special cases". The plan now transfers up to 90 credits if everything posts (57 posted so far), after moving CS 2401, CS 3340 and CS 4408 to Study.com. UoPeople's own Study.com pathway guide (valid 2025-2026) lists 81 transfer credits and 39 UoPeople credits, which already exceeds 50%, so cite it. Ask the Transfer Evaluation contact whether the 75% exception applies BEFORE paying for the remaining Study.com courses. Any course not approved must be retaken at UoPeople ($180 each). No transfer credit beyond 90 counts, so the spare Psychology, Nutrition and extra Google IT credits are surplus.</t>
+          <t>UoPeople's default transfer allowance is 50% of the degree (60 credits / 20 courses). The 75% ceiling (90 credits / 30 courses) is only granted "in special cases". The plan now transfers up to 90 credits if everything posts (57 posted so far), after moving CS 2401, CS 3340 and CS 3307 to Study.com. UoPeople's own Study.com pathway guide (valid 2025-2026) lists 81 transfer credits and 39 UoPeople credits, which already exceeds 50%, so cite it. Ask the Transfer Evaluation contact whether the 75% exception applies BEFORE paying for the remaining Study.com courses. Any course not approved must be retaken at UoPeople ($180 each). No transfer credit beyond 90 counts, so the spare Psychology, Nutrition and extra Google IT credits are surplus.</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="B4" s="47" t="inlineStr">
         <is>
-          <t>Audit of 20 Oct 2026: 57 of 120 credits posted (Major 27/60, General Education 21/30, Electives 9/30). Calculus posted as MATH 1211 (3 of 4 semester hours) and Study.com Networking posted as Major Elective 2 (EXT-MAJ 1002), so CS 3308 is no longer needed. Still not posted: Java (CS 1103, on the published Sophia list, so ask the transfer office) and Public Speaking (Social Science needs 3 credits). Critical Thinking and Project Management are not needed. Discrete Mathematics and Operating Systems 1 are passed and go in the next Study.com request. Still uncovered: COM 2001 (Study.com Business 113, Business 313 or Communications 102) and one Social Science course (Public Speaking if it posts, otherwise Sophia Introduction to Sociology). Remaining: 21 courses, 11 by transfer and 10 direct. The plan lands at exactly 90 transfer credits, so there is no room for an extra transfer course.</t>
+          <t>Audit of 20 Oct 2026: 57 of 120 credits posted (Major 27/60, General Education 21/30, Electives 9/30). Calculus posted as MATH 1211 (3 of 4 semester hours) and Study.com Networking posted as Major Elective 2 (EXT-MAJ 1002), so CS 3308 is no longer needed. Still not posted: Java (CS 1103, on the published Sophia list, so ask the transfer office) and Public Speaking (Social Science needs 3 credits). Critical Thinking and Project Management are not needed. Discrete Mathematics and Operating Systems 1 are passed and go in the next Study.com request. Still uncovered: COM 2001 (Study.com Business 113, Business 313 or Communications 102) and one Social Science course (Public Speaking if it posts, otherwise Sophia Introduction to Sociology). Remaining: 21 courses, 11 by transfer and 10 direct. The plan lands at exactly 90 transfer credits, so there is no room for an extra transfer course. Proctored courses (8 required, 3 posted): Study.com now covers CS 2301, 3303, 3306 and CS 3307 (CS 305). CS 4408 moved back to UoPeople to stay at 90 transfer credits. CS 3305, 4402 and 4407 are proctored with no Study.com equivalent. The only other proctored Study.com course that maps to a UoPeople course is History 101 for HIST 1421, but Civilization Studies is already complete, so it would be surplus credit that uses cap room.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Study.com transcript of 26 Oct: Discrete Math, OS1, Data Structures, Databases 2 submitted
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012zoe9p2gYUKrMz8itSXJDw
</commit_message>
<xml_diff>
--- a/UoPeople_CS_Degree_Roadmap_updated.xlsx
+++ b/UoPeople_CS_Degree_Roadmap_updated.xlsx
@@ -1647,12 +1647,12 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>DONE (not transferred)</t>
+          <t>DONE (submitted 26 Oct)</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Passed 97%. Not on the 13 Oct transcript, so include it in the next request.</t>
+          <t>Passed 97% on 13 Oct. On the Study.com transcript submitted 26 Oct, pending posting.</t>
         </is>
       </c>
     </row>
@@ -1687,12 +1687,12 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>DONE (not transferred)</t>
+          <t>DONE (submitted 26 Oct)</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Passed. Include it in the next request. Proctored at UoPeople.</t>
+          <t>Passed 93% on 14 Oct. On the Study.com transcript submitted 26 Oct, pending posting.</t>
         </is>
       </c>
     </row>
@@ -1767,12 +1767,12 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE (submitted 26 Oct)</t>
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>Month 1. Proctored at UoPeople, so transferring avoids the exam.</t>
+          <t>Passed 95% on 19 Oct. On the Study.com transcript submitted 26 Oct, pending posting.</t>
         </is>
       </c>
     </row>
@@ -1807,12 +1807,12 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE (submitted 26 Oct)</t>
         </is>
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>Month 1. Per the UoPeople/Study.com pathway guide.</t>
+          <t>Passed 96% on 22 Oct. On the Study.com transcript submitted 26 Oct, pending posting.</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="B4" s="47" t="inlineStr">
         <is>
-          <t>Audit of 24 Oct 2026: 60 of 120 credits posted (Major 27/60, General Education 24/30, Electives 9/30). Sociology posted as SOC 1502, so Social Science is complete. Java (CS 1103) is still not posted, ask the transfer office. Public Speaking, Critical Thinking and Project Management are not needed. Still uncovered: COM 2001 (Study.com Business 113, Business 313 or Communications 102) and UNIV 1001 (direct). Remaining: 20 courses, 10 by transfer and 10 direct. The plan lands at exactly 90 transfer credits. Proctored counter is 3/8 (CS 2205, MATH 1201, MATH 1280). The 24 Oct export labels CS 2301, 3303, 3305, 3306, 3307, 4402 and 4407 as non-proctored, while the 20 Oct portal view labelled them proctored. Confirm with the advisor which is correct and what counts toward the 8.</t>
+          <t>Audit of 24 Oct 2026: 60 of 120 credits posted (Major 27/60, General Education 24/30, Electives 9/30). Sociology posted as SOC 1502, so Social Science is complete. Java (CS 1103) is still not posted, ask the transfer office. Public Speaking, Critical Thinking and Project Management are not needed. Still uncovered: COM 2001 (Study.com Business 113, Business 313 or Communications 102) and UNIV 1001 (direct). Remaining: 20 courses, 10 by transfer and 10 direct. The plan lands at exactly 90 transfer credits. Proctored counter is 3/8 (CS 2205, MATH 1201, MATH 1280). The 24 Oct export labels CS 2301, 3303, 3305, 3306, 3307, 4402 and 4407 as non-proctored, while the 20 Oct portal view labelled them proctored. Confirm with the advisor which is correct and what counts toward the 8. Second Study.com transcript submitted 26 Oct: Discrete Mathematics, Operating Systems 1, Data Structures and Databases 2 are new. Calculus and Networking are on it again, already posted.</t>
         </is>
       </c>
     </row>

</xml_diff>